<commit_message>
Update PCB fabrication requirements and harness drawings
</commit_message>
<xml_diff>
--- a/02_PCB/01_FPC柔性板/05_PCBA加工要求_FPC.xlsx
+++ b/02_PCB/01_FPC柔性板/05_PCBA加工要求_FPC.xlsx
@@ -8,8 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="基本信息" sheetId="2" r:id="rId5"/>
-    <sheet name="附图1" sheetId="3" r:id="rId6"/>
-    <sheet name="附图2" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcMode="auto"/>
   <extLst>
@@ -49,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t xml:space="preserve">  </t>
   </si>
@@ -172,9 +170,6 @@
     <t xml:space="preserve">说明：</t>
   </si>
   <si>
-    <t xml:space="preserve">详见附图1</t>
-  </si>
-  <si>
     <t xml:space="preserve">相关标准</t>
   </si>
   <si>
@@ -200,22 +195,6 @@
   </si>
   <si>
     <t xml:space="preserve">不固定自行贴</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOP层100Ω
-差分阻抗匹配</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOT层100Ω
-差分阻抗匹配</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOT层90Ω
-差分阻抗匹配</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIG03层120Ω
-差分阻抗匹配</t>
   </si>
 </sst>
 </file>
@@ -445,7 +424,7 @@
   <cellStyleXfs count="1">
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="24">
     <xf applyAlignment="false" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -517,15 +496,6 @@
     </xf>
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="15" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="center" wrapText="true"/>
-    </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="center" wrapText="true"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -542,155 +512,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>-38100</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>-38100</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2" descr="avhdCT"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="false"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="false" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>-38100</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>-38100</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 3" descr="CrPshV"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="false"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="false" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>-38100</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>-38100</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 4" descr="coLGMX"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="false"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="false" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>-38100</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>-38100</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 5" descr="ptzzRO"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="false"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="false" fPrintsWithSheet="true"/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1150,13 +971,13 @@
       <c r="A12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="12" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1170,7 +991,7 @@
       <c r="C13" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="12" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1184,42 +1005,40 @@
       <c r="C14" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>40</v>
-      </c>
+      <c r="D14" s="14"/>
     </row>
     <row customHeight="true" ht="20" r="15">
       <c r="A15" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="C15" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="13" t="s">
         <v>43</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>44</v>
       </c>
     </row>
     <row customHeight="true" ht="20" r="16">
       <c r="A16" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="C16" s="10"/>
+      <c r="D16" s="12" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="14" t="s">
-        <v>47</v>
       </c>
     </row>
     <row customHeight="true" ht="20" r="17">
       <c r="A17" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="16" t="s">
         <v>48</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>49</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>39</v>
@@ -2333,9 +2152,6 @@
     <mergeCell ref="B18:D19"/>
   </mergeCells>
   <dataValidations count="9">
-    <dataValidation allowBlank="true" errorStyle="stop" showErrorMessage="true" sqref="D7:D7" type="list">
-      <formula1>"白色,黑色"</formula1>
-    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" showErrorMessage="true" sqref="B9:B9" type="list">
       <formula1>"按GERBER,按PCB文件"</formula1>
     </dataValidation>
@@ -2345,8 +2161,8 @@
     <dataValidation allowBlank="true" errorStyle="stop" showErrorMessage="true" sqref="B16:B16" type="list">
       <formula1>"不拼板,供应商自行拼板,自定义"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" showErrorMessage="true" sqref="B4:B4" type="list">
-      <formula1>"2,4,6,8,10,12"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" showErrorMessage="true" sqref="D7:D7" type="list">
+      <formula1>"白色,黑色"</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" showErrorMessage="true" sqref="B8:B8" type="list">
       <formula1>"按合同数量,自定义"</formula1>
@@ -2360,75 +2176,12 @@
     <dataValidation allowBlank="true" errorStyle="stop" showErrorMessage="true" sqref="B17:B17" type="list">
       <formula1>"不固定自行贴,固定Label区域"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" showErrorMessage="true" sqref="B4:B4" type="list">
+      <formula1>"2,4,6,8,10,12"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100"/>
   <picture r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{00000000-0001-0000-0000-000000000000}" mc:Ignorable="x14ac xr xr2 xr3 xr6 xr10 x15">
-  <sheetPr>
-    <outlinePr summaryBelow="false" summaryRight="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="60.0909090909091"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="2" min="2" style="0" width="21"/>
-  </cols>
-  <sheetData>
-    <row customHeight="true" ht="360" r="1">
-      <c r="A1" s="24"/>
-      <c r="B1" s="25" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row customHeight="true" ht="365" r="2">
-      <c r="A2" s="24"/>
-      <c r="B2" s="25" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="24"/>
-      <c r="B3" s="25" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="24"/>
-      <c r="B4" s="25" t="s">
-        <v>53</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100"/>
-  <drawing r:id="rId1"/>
-  <picture r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{00000000-0001-0000-0000-000000000000}" mc:Ignorable="x14ac xr xr2 xr3 xr6 xr10 x15">
-  <sheetPr>
-    <outlinePr summaryBelow="false" summaryRight="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="54.9090909090909"/>
-  </cols>
-  <sheetData>
-    <row customHeight="true" ht="230" r="1"/>
-    <row customHeight="true" ht="53" r="2">
-      <c r="A2" s="26"/>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100"/>
-  <picture r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>